<commit_message>
Update master data with new DAF values
</commit_message>
<xml_diff>
--- a/data/inputs/Artikel & Materialien FGR+.XLSX
+++ b/data/inputs/Artikel & Materialien FGR+.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uklra\Downloads\ddmrp_mvp_monorepo\backend\data\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8105D042-DB35-4C61-8DC1-031FEE796F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C68ABF2-8110-4F98-B7B2-152C99CF12F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1084,7 +1084,7 @@
         <v>19</v>
       </c>
       <c r="C21" s="2">
-        <v>1.9</v>
+        <v>1</v>
       </c>
       <c r="D21" s="2">
         <v>4</v>

</xml_diff>